<commit_message>
docs(2359): update post-Q4 catalyst, add MTP track record analysis
- FY3/26 OP ¥3.82B, +9% above revised MTP target
- Add 3-MTP OP growth history (12th/13th/14th)
- Note FY3/26 target downward revision (April 28, 2025 footnote)
- Update next catalyst to 15th MTP announcement
- Refresh models/2359_DCF_Model_20260410.xlsx with post-Q4 data
</commit_message>
<xml_diff>
--- a/models/2359_DCF_Model_20260410.xlsx
+++ b/models/2359_DCF_Model_20260410.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ryosuke0923\ryosuke-japanese-equity-research\models\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{765CDE1A-2CA1-45E3-BF58-A691B7403B73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA4A81DC-5F40-44B9-AC9A-2A5A04F9DAE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Executive Summary" sheetId="1" r:id="rId1"/>
@@ -1328,7 +1328,7 @@
         <v>9</v>
       </c>
       <c r="C9" s="5">
-        <v>2252</v>
+        <v>2011</v>
       </c>
     </row>
     <row r="10" spans="2:5" ht="14" x14ac:dyDescent="0.3">
@@ -1355,7 +1355,7 @@
       </c>
       <c r="C12" s="7">
         <f>(C10-C9)/C9</f>
-        <v>0.23090586145648312</v>
+        <v>0.37841869716558924</v>
       </c>
     </row>
     <row r="14" spans="2:5" ht="14" x14ac:dyDescent="0.3">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="D16" s="7">
         <f>(C16-C9)/C9</f>
-        <v>0.26998223801065718</v>
+        <v>0.42217802088513179</v>
       </c>
     </row>
     <row r="17" spans="2:4" ht="13.5" x14ac:dyDescent="0.25">
@@ -1399,7 +1399,7 @@
       </c>
       <c r="D17" s="7">
         <f>(C17-C9)/C9</f>
-        <v>0.66829484902309055</v>
+        <v>0.86822476379910496</v>
       </c>
     </row>
     <row r="18" spans="2:4" ht="13.5" x14ac:dyDescent="0.25">
@@ -1412,7 +1412,7 @@
       </c>
       <c r="D18" s="7">
         <f>(C18-C9)/C9</f>
-        <v>8.7921847246891657E-2</v>
+        <v>0.21829935355544505</v>
       </c>
     </row>
     <row r="19" spans="2:4" ht="13.5" x14ac:dyDescent="0.25">
@@ -1425,7 +1425,7 @@
       </c>
       <c r="D19" s="7">
         <f>(C19-C9)/C9</f>
-        <v>-0.10257548845470693</v>
+        <v>4.9726504226752857E-3</v>
       </c>
     </row>
     <row r="21" spans="2:4" ht="14" x14ac:dyDescent="0.3">

</xml_diff>